<commit_message>
docs(article): fix Overview link, remove Held status, trim user-facing statuses
Point the product link at intainft.com/intainmarkets, rename role headings to
Issuer or Borrower style, drop HELD/Inactive/backend-only statuses, and use
Transferred / Retirement pending / Retired for NFT lifecycle docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
+++ b/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale product line, updated platform positioning to include all four product lines and blockchain settlement capabilities</t>
+          <t>Modified — Fixed Overview product link to https://intainft.com/intainmarkets; role headings Issuers or Borrowers / Market Makers or Facility Agents / Investors or Lenders; removed HELD from NFT lifecycle</t>
         </is>
       </c>
     </row>
@@ -1442,9 +1442,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="G34" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article documenting all Asset Sale deal statuses and transitions</t>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed HELD and Inactive; NFT statuses use Transferred / Retirement pending / Retired; trimmed backend rail statuses</t>
         </is>
       </c>
     </row>
@@ -1523,9 +1523,9 @@
           <t>K</t>
         </is>
       </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article with detailed settlement mechanics, all payment rails, and NFT transfer</t>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed HELD and backend rail/lock statuses; user-facing settlement + NFT statuses only</t>
         </is>
       </c>
     </row>
@@ -1550,9 +1550,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for the end-to-end repayment process</t>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Modified — NFT lifecycle without HELD; user-facing Retirement pending / Retired labels</t>
         </is>
       </c>
     </row>
@@ -2295,9 +2295,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G65" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Investor's repayment confirmation and NFT burn</t>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Replaced BURN_PENDING/BURNED with Retirement pending / Retired</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale composite statuses and qualifier vocabulary</t>
+          <t>Modified — Removed Inactive from deal status qualifiers</t>
         </is>
       </c>
     </row>
@@ -2485,9 +2485,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="G71" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Asset Sale status definitions and CTA mapping</t>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed HELD/Inactive/Settled Late; user-facing deal/settlement/NFT statuses only; added Approved</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added status renames, Settlement v2, e-signature migration, API consolidation</t>
+          <t>Modified — Terminal statuses no longer include Inactive; added Approved to lifecycle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(article): rewrite guides in plain user language and apply repayment review fixes
Clarify Intain loan-tape help, drop internal repayment fields and duplicate tables, and remove backend status codes and field names from the knowledge base.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
+++ b/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
@@ -49,7 +49,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -93,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +122,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -618,7 +626,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for Entra SSO login flow, added Asset Sale navigation sections, updated sidebar menu structure</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -645,7 +653,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Modified — Extended philosophy to cover Asset Sale deal statuses and settlement approval gates</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -707,7 +715,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Modified — Clarified status transition triggers and role-based actions at each state</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -802,7 +810,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>What loans represent in the platform — individual receivables within pools. Covers loan onboarding (Loan Registry v2), batch verification via Verification Agent (ABDP integration), NFT minting for receivables, and loan data fields.</t>
+          <t>What loans represent in the platform — individual receivables within pools. Covers upload, field matching, the Loan Registry, batch verification (self-certify or a verification agent), and NFT minting.</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
@@ -815,7 +823,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Loan Registry v2, batch verification, ABDP integration, and receivables NFT minting details</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -842,7 +850,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Modified — Enhanced status explanations with trigger conditions and calculation impact</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -968,7 +976,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>End-to-end credit facility lifecycle — from term sheet negotiation through master commitment creation, facility setup (RemoteV2 11-tab wizard), funding requests, token generation, e-signature, and settlement. Covers the complete Borrower → Facility Agent → Lender workflow.</t>
+          <t>End-to-end credit facility lifecycle — from term sheet through master commitment, deal setup, funding requests, funding notices, and lender confirmation of funds.</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
@@ -981,7 +989,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added RemoteV2 creation wizard details, updated lifecycle to reflect current flow</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1006,9 +1014,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1043,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Modified — Enhanced field descriptions and validation rules</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1060,9 +1068,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1087,9 +1095,9 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1114,9 +1122,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1138,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Two-phase facility setup tracking: 'In Progress' (RemoteV2 wizard tabs being completed) vs. 'Completed' (all required tabs filled, facility ready for operations). Explains which tabs are mandatory and validation requirements.</t>
+          <t>Facility setup status: In Progress while deal modelling is unfinished, and Completed when borrowers can map loans and create funding requests.</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
@@ -1143,7 +1151,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for RemoteV2 11-tab wizard, clarified mandatory tab requirements</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1168,9 +1176,9 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1195,9 +1203,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1222,9 +1230,9 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1313,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for Adobe Sign + ZohoSign, noted DocuSign deprecation</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1330,9 +1338,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1357,9 +1365,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1384,9 +1392,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1415,9 +1423,9 @@
           <t>J</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for the Asset Sale product line, covering the complete WLS concept and lifecycle</t>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1452,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed HELD and Inactive; NFT statuses use Transferred / Retirement pending / Retired; trimmed backend rail statuses</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1469,9 +1477,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for the Issuer deal creation wizard</t>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1496,9 +1504,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for investor commitment and allocation workflow</t>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1533,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed HELD and backend rail/lock statuses; user-facing settlement + NFT statuses only</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1560,7 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Modified — NFT lifecycle without HELD; user-facing Retirement pending / Retired labels</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1577,9 +1585,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for NFT burn mechanics and deal closure</t>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1604,9 +1612,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Asset Sale analytics and performance tracking</t>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1631,9 +1639,9 @@
           <t>K</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Asset Sale e-signature workflow</t>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1720,9 +1728,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1747,9 +1755,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1774,9 +1782,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1801,9 +1809,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Issuer's Asset Sale deal setup workflow</t>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1828,9 +1836,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Issuer's repayment initiation process</t>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1886,9 +1894,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1923,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for RemoteV2 11-tab creation wizard</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1977,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added syntax examples and common pattern library</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2031,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added borrowing base and covenant compliance checks</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2058,7 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for Adobe Sign + ZohoSign, removed DocuSign references</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2075,9 +2083,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G57" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Underwriter's Asset Sale management workflow</t>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2133,9 +2141,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2268,9 +2276,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G64" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Investor's Asset Sale participation workflow</t>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2305,7 @@
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Modified — Replaced BURN_PENDING/BURNED with Retirement pending / Retired</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2340,7 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added 'In Deal' and 'Closed' states, enhanced trigger descriptions</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2392,9 +2400,9 @@
           <t>E</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2433,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed Inactive from deal status qualifiers</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2464,7 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale actions and deal-level CTA states</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2495,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed HELD/Inactive/Settled Late; user-facing deal/settlement/NFT statuses only; added Approved</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2530,7 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Modified — Extended to cover Asset Sale approval gates (Underwriter review, settlement confirmation)</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2561,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale deal rejection scenarios</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2582,9 +2590,9 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2623,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added complete Asset Sale permissions matrix for Issuer, Underwriter, Investor, Servicer</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2658,7 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added centralized audit module details, blockchain traceability, export capabilities</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2689,7 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added centralized audit module view reference</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2720,7 @@
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for Adobe Sign + ZohoSign, removed DocuSign references</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2751,7 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Modified — Updated for Avalanche L1 subnet, added burn event evidence</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2782,7 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added MFA, rate limiting, Entra SSO, admin impersonation controls</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2848,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added settlement comparison and cross-product-line FAQs</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2879,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale blocking reasons and resolution steps</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2910,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added role-status matrix and View As limitations</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2931,9 +2939,9 @@
           <t>H</t>
         </is>
       </c>
-      <c r="G85" s="8" t="inlineStr">
-        <is>
-          <t>Created — New article for Asset Sale-specific frequently asked questions</t>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2963,7 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Chronological log of all new features added to the platform — Asset Sale product line, Entra SSO, centralized Audit Module, v2 API consolidation (pools, loans, batches, orgs, users, dataroom), Modelling Workbench, Historical Tape upload, Batches v2, Loan Registry v2, wallet onboarding updates, and more.</t>
+          <t>New platform capabilities — Asset Sale, Microsoft sign-in, Activity Audit, Adobe Sign and ZohoSign, Participation Agreements, notifications, and list search.</t>
         </is>
       </c>
       <c r="E86" s="6" t="n">
@@ -2968,7 +2976,7 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added all features since January 2026 (Asset Sale, Entra SSO, Audit Module, v2 APIs, etc.)</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2994,7 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Record of all workflow and status changes — WLS status vocabulary renames (Closed → Active, Repaid → Closed), Settlement v2 unified engine, e-signature provider migration (DocuSign deprecated, Adobe Sign + ZohoSign adopted), and API route consolidation from v1 to v2.</t>
+          <t>Status and workflow changes — asset sale Closed now means a finished repayment and Active means a settled sale, plus Adobe Sign and ZohoSign, Microsoft sign-in, and Activity Audit.</t>
         </is>
       </c>
       <c r="E87" s="6" t="n">
@@ -2999,7 +3007,7 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Modified — Terminal statuses no longer include Inactive; added Approved to lifecycle</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3025,7 @@
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Record of all retired platform capabilities — legacy v1 API routes replaced by v2, DocuSign e-signature removed (replaced by Adobe Sign + ZohoSign), IPFS storage retired, and any deprecated UI flows or features that users should no longer reference.</t>
+          <t>Retired or replaced capabilities — DocuSign replaced by Adobe Sign and ZohoSign, older files still open, notifications and the data room updated, and NFT minting moved to Certificates.</t>
         </is>
       </c>
       <c r="E88" s="6" t="n">
@@ -3030,7 +3038,7 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added DocuSign deprecation, IPFS retirement, v1 API deprecation details</t>
+          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(article): compact all articles to short concise guides
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
+++ b/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Modified — Fixed Overview product link to https://intainft.com/intainmarkets; role headings Issuers or Borrowers / Market Makers or Facility Agents / Investors or Lenders; removed HELD from NFT lifecycle</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Underwriter/Facility Agent aliases for Market Maker, added Verification Agent and Rating Agency roles, expanded Asset Sale role permissions</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added connection to Asset Sale deals, updated pool analysis IDA integration details</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale context for pool views, clarified Underwriter view</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Modified — Enhanced step-by-step detail, added notification flow description</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added attention indicator details and iteration cycle explanation</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added impact on deal calculations and investor allocations</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Modified — Enhanced field-by-field guidance, added common pitfalls section</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added cascade impact explanation for loan changes</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added evaluation best practices and loan quality metrics guidance</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added IDA analytics integration and risk metrics</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2249,9 +2249,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged</t>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added calculation impact and visibility rules per role</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale, audit module, and Entra SSO FAQs</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Condensed to short-form concise guide</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(article): fix roles, sidebar, terminology, FAQ format, content completeness
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
+++ b/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Modified — Added Asset Sale Receivables analytics, expanded IDA Pool Analysis capabilities</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Modified — Condensed to short-form concise guide</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Modified — Removed internal field names and system status codes; rewritten in plain language for platform users</t>
+          <t>Modified — Terminology fix, content completeness review, flow order</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(article): add Securitization module documentation (articles 88-95)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
+++ b/Intain Markets – Knowledge Base Categories & Sub-Categories.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +127,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3042,6 +3043,258 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>Securitization</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>Module Overview</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>Securitization Overview</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>Introduction to the Securitization product line — pool-to-deal conversion, tranches, FT tokens, commit/invest phases, roles, and payment modes.</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="G89" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="n"/>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Deal Lifecycle</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>Securitization Deal Lifecycle &amp; Statuses</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>Deal statuses (Created, Awaiting Approval, Open, Closed), tranche approval statuses (Pending, Approved, Rejected), and commit vs invest phase definitions.</t>
+        </is>
+      </c>
+      <c r="E90" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G90" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="n"/>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>Deal Creation</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>Deal Creation &amp; Tranche Setup</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="inlineStr">
+        <is>
+          <t>Step-by-step guide to creating a securitization deal from a pool and adding tranches — required fields, FT contract deployment, and deal approval flow.</t>
+        </is>
+      </c>
+      <c r="E91" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G91" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n"/>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Investor Workflows</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>Investor Commitment Phase</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>Investor commit workflow — selecting tranches, entering commit amounts, available commitment calculations, and validation rules including one-commitment-per-tranche enforcement.</t>
+        </is>
+      </c>
+      <c r="E92" s="10" t="n">
+        <v>91</v>
+      </c>
+      <c r="F92" s="10" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G92" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="n"/>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>Investor Workflows</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>Investment &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>Invest phase workflow for investors — offchain (bank wire) and onchain (USDC/MetaMask) settlement flows, settlement record creation, and post-investment FT delivery trigger.</t>
+        </is>
+      </c>
+      <c r="E93" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="F93" s="10" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G93" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="n"/>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Token Delivery</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>Token Approval &amp; FT Delivery</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr">
+        <is>
+          <t>Issuer FT contract approval (MFA + on-chain signing) and Paying Agent FT delivery (MFA) per tranche — delivery to one investor or all investors.</t>
+        </is>
+      </c>
+      <c r="E94" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="F94" s="10" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G94" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n"/>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>Accounts &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>Accounts &amp; Transactions</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>Reference for deal account types (Closing, Principal Remittance, Interest Remittance, Collateral Balance), transaction ledger fields, ending balance calculation, and ESMA reporting link.</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="F95" s="10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="G95" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n"/>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Roles &amp; Permissions</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>Securitization Roles &amp; Permissions</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="inlineStr">
+        <is>
+          <t>Complete permissions matrix for Securitization — role actions by deal status, phase-gated restrictions, one-commitment enforcement, and MFA requirements for Issuer and Paying Agent.</t>
+        </is>
+      </c>
+      <c r="E96" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="F96" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G96" s="10" t="inlineStr">
+        <is>
+          <t>Created — New Securitization module documentation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>